<commit_message>
fix style bug in ExportExcelPackagePassport
</commit_message>
<xml_diff>
--- a/data/Excel/prikaz_package_passport.xlsx
+++ b/data/Excel/prikaz_package_passport.xlsx
@@ -617,7 +617,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -695,12 +695,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -880,70 +917,37 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -961,12 +965,12 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -976,22 +980,61 @@
     <xf numFmtId="0" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1327,29 +1370,29 @@
       <c r="G3" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="100"/>
-      <c r="I3" s="101"/>
-      <c r="J3" s="101"/>
+      <c r="H3" s="89"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
       <c r="K3" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="L3" s="102"/>
-      <c r="M3" s="103"/>
+      <c r="L3" s="91"/>
+      <c r="M3" s="92"/>
       <c r="N3"/>
       <c r="T3" s="31"/>
       <c r="U3" s="31"/>
       <c r="V3" s="31"/>
     </row>
     <row r="4" spans="1:22" s="5" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H4" s="113" t="s">
+      <c r="H4" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="I4" s="113"/>
-      <c r="J4" s="113"/>
-      <c r="L4" s="114" t="s">
+      <c r="I4" s="80"/>
+      <c r="J4" s="80"/>
+      <c r="L4" s="81" t="s">
         <v>3</v>
       </c>
-      <c r="M4" s="114"/>
+      <c r="M4" s="81"/>
       <c r="T4" s="25" t="s">
         <v>50</v>
       </c>
@@ -1361,11 +1404,11 @@
       <c r="H5" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="104"/>
-      <c r="J5" s="105"/>
-      <c r="K5" s="105"/>
-      <c r="L5" s="105"/>
-      <c r="M5" s="105"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="94"/>
+      <c r="K5" s="94"/>
+      <c r="L5" s="94"/>
+      <c r="M5" s="94"/>
       <c r="T5" s="19">
         <v>1</v>
       </c>
@@ -1375,13 +1418,13 @@
     <row r="6" spans="1:22" s="7" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G6" s="43"/>
       <c r="H6" s="43"/>
-      <c r="I6" s="106" t="s">
+      <c r="I6" s="82" t="s">
         <v>5</v>
       </c>
-      <c r="J6" s="107"/>
-      <c r="K6" s="107"/>
-      <c r="L6" s="107"/>
-      <c r="M6" s="107"/>
+      <c r="J6" s="95"/>
+      <c r="K6" s="95"/>
+      <c r="L6" s="95"/>
+      <c r="M6" s="95"/>
       <c r="T6" s="19">
         <v>2</v>
       </c>
@@ -1392,11 +1435,11 @@
       <c r="H7" s="67" t="s">
         <v>70</v>
       </c>
-      <c r="I7" s="108"/>
-      <c r="J7" s="108"/>
-      <c r="K7" s="108"/>
-      <c r="L7" s="108"/>
-      <c r="M7" s="108"/>
+      <c r="I7" s="97"/>
+      <c r="J7" s="97"/>
+      <c r="K7" s="97"/>
+      <c r="L7" s="97"/>
+      <c r="M7" s="97"/>
       <c r="T7" s="19">
         <v>3</v>
       </c>
@@ -1413,18 +1456,18 @@
       <c r="B9" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="93"/>
-      <c r="D9" s="94"/>
+      <c r="C9" s="103"/>
+      <c r="D9" s="104"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-      <c r="G9" s="95"/>
-      <c r="H9" s="95"/>
-      <c r="I9" s="95"/>
+      <c r="G9" s="96"/>
+      <c r="H9" s="96"/>
+      <c r="I9" s="96"/>
       <c r="J9" s="45"/>
       <c r="K9" s="45"/>
       <c r="L9" s="45"/>
-      <c r="M9" s="95"/>
-      <c r="N9" s="95"/>
+      <c r="M9" s="96"/>
+      <c r="N9" s="96"/>
       <c r="O9" s="74"/>
       <c r="P9" s="74" t="s">
         <v>73</v>
@@ -1450,20 +1493,20 @@
       <c r="D10" s="47"/>
       <c r="E10" s="46"/>
       <c r="F10" s="46"/>
-      <c r="G10" s="114" t="s">
+      <c r="G10" s="81" t="s">
         <v>6</v>
       </c>
-      <c r="H10" s="114"/>
-      <c r="I10" s="114"/>
+      <c r="H10" s="81"/>
+      <c r="I10" s="81"/>
       <c r="J10" s="46"/>
       <c r="K10" s="46"/>
       <c r="L10" s="46"/>
-      <c r="M10" s="114" t="s">
+      <c r="M10" s="81" t="s">
         <v>71</v>
       </c>
-      <c r="N10" s="114"/>
-      <c r="O10" s="114"/>
-      <c r="P10" s="114"/>
+      <c r="N10" s="81"/>
+      <c r="O10" s="81"/>
+      <c r="P10" s="81"/>
       <c r="Q10" s="46"/>
       <c r="R10" s="46"/>
       <c r="S10" s="46"/>
@@ -1509,15 +1552,15 @@
       <c r="G12" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="H12" s="96"/>
-      <c r="I12" s="96"/>
-      <c r="J12" s="96"/>
+      <c r="H12" s="105"/>
+      <c r="I12" s="105"/>
+      <c r="J12" s="105"/>
       <c r="K12" s="75"/>
       <c r="L12" s="45"/>
-      <c r="M12" s="95"/>
-      <c r="N12" s="95"/>
-      <c r="O12" s="95"/>
-      <c r="P12" s="95"/>
+      <c r="M12" s="96"/>
+      <c r="N12" s="96"/>
+      <c r="O12" s="96"/>
+      <c r="P12" s="96"/>
       <c r="Q12" s="51"/>
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
@@ -1533,19 +1576,19 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
-      <c r="H13" s="106" t="s">
+      <c r="H13" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="I13" s="106"/>
-      <c r="J13" s="106"/>
-      <c r="K13" s="115"/>
+      <c r="I13" s="82"/>
+      <c r="J13" s="82"/>
+      <c r="K13" s="83"/>
       <c r="L13" s="45"/>
-      <c r="M13" s="106" t="s">
+      <c r="M13" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="N13" s="106"/>
-      <c r="O13" s="106"/>
-      <c r="P13" s="106"/>
+      <c r="N13" s="82"/>
+      <c r="O13" s="82"/>
+      <c r="P13" s="82"/>
       <c r="Q13" s="51"/>
       <c r="R13" s="48"/>
       <c r="S13" s="55"/>
@@ -1563,17 +1606,17 @@
       <c r="G14" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="H14" s="92"/>
-      <c r="I14" s="92"/>
-      <c r="J14" s="92"/>
-      <c r="K14" s="92"/>
-      <c r="L14" s="92"/>
+      <c r="H14" s="102"/>
+      <c r="I14" s="102"/>
+      <c r="J14" s="102"/>
+      <c r="K14" s="102"/>
+      <c r="L14" s="102"/>
       <c r="M14" s="76" t="s">
         <v>74</v>
       </c>
-      <c r="N14" s="92"/>
-      <c r="O14" s="92"/>
-      <c r="P14" s="92"/>
+      <c r="N14" s="102"/>
+      <c r="O14" s="102"/>
+      <c r="P14" s="102"/>
       <c r="Q14" s="57"/>
       <c r="R14" s="57"/>
       <c r="S14" s="1"/>
@@ -1591,17 +1634,17 @@
       <c r="G15" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="97"/>
-      <c r="I15" s="97"/>
-      <c r="J15" s="97"/>
-      <c r="K15" s="97"/>
-      <c r="L15" s="97"/>
+      <c r="H15" s="106"/>
+      <c r="I15" s="106"/>
+      <c r="J15" s="106"/>
+      <c r="K15" s="106"/>
+      <c r="L15" s="106"/>
       <c r="M15" s="76" t="s">
         <v>74</v>
       </c>
-      <c r="N15" s="92"/>
-      <c r="O15" s="92"/>
-      <c r="P15" s="92"/>
+      <c r="N15" s="102"/>
+      <c r="O15" s="102"/>
+      <c r="P15" s="102"/>
       <c r="Q15" s="58"/>
       <c r="R15" s="58"/>
       <c r="S15" s="58"/>
@@ -1619,17 +1662,17 @@
       <c r="G16" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="95"/>
-      <c r="I16" s="95"/>
-      <c r="J16" s="95"/>
+      <c r="H16" s="96"/>
+      <c r="I16" s="96"/>
+      <c r="J16" s="96"/>
       <c r="K16" s="59"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="O16" s="98"/>
-      <c r="P16" s="98"/>
+      <c r="O16" s="100"/>
+      <c r="P16" s="100"/>
       <c r="Q16" s="1"/>
       <c r="R16" s="60"/>
       <c r="S16" s="1"/>
@@ -1675,17 +1718,17 @@
       <c r="G18" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="H18" s="99"/>
-      <c r="I18" s="95"/>
-      <c r="J18" s="99"/>
+      <c r="H18" s="101"/>
+      <c r="I18" s="96"/>
+      <c r="J18" s="101"/>
       <c r="K18" s="53"/>
       <c r="L18" s="45"/>
       <c r="M18" s="45"/>
       <c r="N18" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="O18" s="98"/>
-      <c r="P18" s="98"/>
+      <c r="O18" s="100"/>
+      <c r="P18" s="100"/>
       <c r="Q18" s="45"/>
       <c r="R18" s="53"/>
       <c r="S18" s="54"/>
@@ -1721,60 +1764,60 @@
       <c r="A20" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="109" t="s">
+      <c r="B20" s="98" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="109"/>
-      <c r="D20" s="109"/>
-      <c r="E20" s="109"/>
-      <c r="F20" s="109"/>
-      <c r="G20" s="109"/>
-      <c r="H20" s="109"/>
-      <c r="I20" s="109"/>
-      <c r="J20" s="109"/>
-      <c r="K20" s="109"/>
-      <c r="L20" s="109"/>
-      <c r="M20" s="109"/>
-      <c r="N20" s="109"/>
-      <c r="O20" s="109"/>
-      <c r="P20" s="109"/>
-      <c r="Q20" s="109"/>
-      <c r="R20" s="109"/>
-      <c r="S20" s="109"/>
+      <c r="C20" s="98"/>
+      <c r="D20" s="98"/>
+      <c r="E20" s="98"/>
+      <c r="F20" s="98"/>
+      <c r="G20" s="98"/>
+      <c r="H20" s="98"/>
+      <c r="I20" s="98"/>
+      <c r="J20" s="98"/>
+      <c r="K20" s="98"/>
+      <c r="L20" s="98"/>
+      <c r="M20" s="98"/>
+      <c r="N20" s="98"/>
+      <c r="O20" s="98"/>
+      <c r="P20" s="98"/>
+      <c r="Q20" s="98"/>
+      <c r="R20" s="98"/>
+      <c r="S20" s="98"/>
       <c r="T20" s="13"/>
       <c r="U20" s="13"/>
       <c r="V20" s="13"/>
     </row>
     <row r="21" spans="1:22" s="9" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="110" t="s">
+      <c r="A21" s="99" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="110"/>
-      <c r="C21" s="110"/>
-      <c r="D21" s="110"/>
-      <c r="E21" s="110"/>
-      <c r="F21" s="110"/>
-      <c r="G21" s="110"/>
-      <c r="H21" s="110"/>
-      <c r="I21" s="110" t="s">
+      <c r="B21" s="99"/>
+      <c r="C21" s="99"/>
+      <c r="D21" s="99"/>
+      <c r="E21" s="99"/>
+      <c r="F21" s="99"/>
+      <c r="G21" s="99"/>
+      <c r="H21" s="99"/>
+      <c r="I21" s="99" t="s">
         <v>20</v>
       </c>
-      <c r="J21" s="110"/>
-      <c r="K21" s="110"/>
-      <c r="L21" s="110"/>
-      <c r="M21" s="85" t="s">
+      <c r="J21" s="99"/>
+      <c r="K21" s="99"/>
+      <c r="L21" s="99"/>
+      <c r="M21" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="N21" s="85"/>
-      <c r="O21" s="85" t="s">
+      <c r="N21" s="88"/>
+      <c r="O21" s="88" t="s">
         <v>22</v>
       </c>
-      <c r="P21" s="85"/>
-      <c r="Q21" s="85" t="s">
+      <c r="P21" s="88"/>
+      <c r="Q21" s="88" t="s">
         <v>64</v>
       </c>
-      <c r="R21" s="85"/>
-      <c r="S21" s="85" t="s">
+      <c r="R21" s="88"/>
+      <c r="S21" s="88" t="s">
         <v>65</v>
       </c>
       <c r="T21" s="12" t="s">
@@ -1784,55 +1827,55 @@
       <c r="V21" s="13"/>
     </row>
     <row r="22" spans="1:22" s="9" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="85" t="s">
+      <c r="A22" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="85" t="s">
+      <c r="B22" s="88" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="85"/>
-      <c r="D22" s="85"/>
-      <c r="E22" s="85"/>
-      <c r="F22" s="85"/>
-      <c r="G22" s="85" t="s">
+      <c r="C22" s="88"/>
+      <c r="D22" s="88"/>
+      <c r="E22" s="88"/>
+      <c r="F22" s="88"/>
+      <c r="G22" s="88" t="s">
         <v>25</v>
       </c>
-      <c r="H22" s="85" t="s">
+      <c r="H22" s="88" t="s">
         <v>26</v>
       </c>
-      <c r="I22" s="85" t="s">
+      <c r="I22" s="88" t="s">
         <v>27</v>
       </c>
-      <c r="J22" s="85" t="s">
+      <c r="J22" s="88" t="s">
         <v>28</v>
       </c>
-      <c r="K22" s="85" t="s">
+      <c r="K22" s="88" t="s">
         <v>29</v>
       </c>
-      <c r="L22" s="85" t="s">
+      <c r="L22" s="88" t="s">
         <v>30</v>
       </c>
-      <c r="M22" s="85" t="s">
+      <c r="M22" s="88" t="s">
         <v>59</v>
       </c>
-      <c r="N22" s="85" t="s">
+      <c r="N22" s="88" t="s">
         <v>31</v>
       </c>
-      <c r="O22" s="85"/>
-      <c r="P22" s="85"/>
-      <c r="Q22" s="85"/>
-      <c r="R22" s="85"/>
-      <c r="S22" s="85"/>
+      <c r="O22" s="88"/>
+      <c r="P22" s="88"/>
+      <c r="Q22" s="88"/>
+      <c r="R22" s="88"/>
+      <c r="S22" s="88"/>
       <c r="T22" s="20"/>
       <c r="U22" s="19"/>
       <c r="V22" s="19"/>
     </row>
     <row r="23" spans="1:22" s="10" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="85"/>
-      <c r="B23" s="85" t="s">
+      <c r="A23" s="88"/>
+      <c r="B23" s="88" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="85"/>
+      <c r="C23" s="88"/>
       <c r="D23" s="68" t="s">
         <v>33</v>
       </c>
@@ -1842,23 +1885,23 @@
       <c r="F23" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="G23" s="85"/>
-      <c r="H23" s="85"/>
-      <c r="I23" s="85"/>
-      <c r="J23" s="85"/>
-      <c r="K23" s="85"/>
-      <c r="L23" s="85"/>
-      <c r="M23" s="85"/>
-      <c r="N23" s="85"/>
+      <c r="G23" s="88"/>
+      <c r="H23" s="88"/>
+      <c r="I23" s="88"/>
+      <c r="J23" s="88"/>
+      <c r="K23" s="88"/>
+      <c r="L23" s="88"/>
+      <c r="M23" s="88"/>
+      <c r="N23" s="88"/>
       <c r="O23" s="68">
         <v>0.1</v>
       </c>
       <c r="P23" s="68">
         <v>1</v>
       </c>
-      <c r="Q23" s="85"/>
-      <c r="R23" s="85"/>
-      <c r="S23" s="85"/>
+      <c r="Q23" s="88"/>
+      <c r="R23" s="88"/>
+      <c r="S23" s="88"/>
       <c r="T23" s="24">
         <v>7180</v>
       </c>
@@ -1874,10 +1917,10 @@
       <c r="A24" s="68">
         <v>1</v>
       </c>
-      <c r="B24" s="85">
+      <c r="B24" s="88">
         <v>2</v>
       </c>
-      <c r="C24" s="85"/>
+      <c r="C24" s="88"/>
       <c r="D24" s="68">
         <v>3</v>
       </c>
@@ -1917,10 +1960,10 @@
       <c r="P24" s="68">
         <v>15</v>
       </c>
-      <c r="Q24" s="85">
+      <c r="Q24" s="88">
         <v>16</v>
       </c>
-      <c r="R24" s="85"/>
+      <c r="R24" s="88"/>
       <c r="S24" s="68">
         <v>17</v>
       </c>
@@ -1974,55 +2017,55 @@
       <c r="S26" s="72"/>
     </row>
     <row r="27" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="91" t="s">
+      <c r="A27" s="84" t="s">
         <v>67</v>
       </c>
-      <c r="B27" s="91"/>
-      <c r="C27" s="91"/>
+      <c r="B27" s="84"/>
+      <c r="C27" s="84"/>
       <c r="D27" s="72"/>
       <c r="E27" s="72"/>
       <c r="F27" s="72"/>
-      <c r="G27" s="91"/>
-      <c r="H27" s="91"/>
-      <c r="I27" s="91"/>
-      <c r="J27" s="91"/>
-      <c r="K27" s="91"/>
-      <c r="L27" s="91"/>
-      <c r="M27" s="91"/>
-      <c r="N27" s="91"/>
-      <c r="O27" s="91" t="s">
+      <c r="G27" s="84"/>
+      <c r="H27" s="84"/>
+      <c r="I27" s="84"/>
+      <c r="J27" s="84"/>
+      <c r="K27" s="84"/>
+      <c r="L27" s="84"/>
+      <c r="M27" s="84"/>
+      <c r="N27" s="84"/>
+      <c r="O27" s="84" t="s">
         <v>68</v>
       </c>
-      <c r="P27" s="91"/>
-      <c r="Q27" s="116"/>
-      <c r="R27" s="116"/>
-      <c r="S27" s="116"/>
+      <c r="P27" s="84"/>
+      <c r="Q27" s="85"/>
+      <c r="R27" s="85"/>
+      <c r="S27" s="85"/>
       <c r="T27" s="11"/>
       <c r="U27" s="11"/>
       <c r="V27" s="11"/>
     </row>
     <row r="28" spans="1:22" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="86" t="s">
+      <c r="A28" s="110" t="s">
         <v>60</v>
       </c>
-      <c r="B28" s="87"/>
-      <c r="C28" s="87"/>
-      <c r="D28" s="87"/>
-      <c r="E28" s="87"/>
-      <c r="F28" s="87"/>
-      <c r="G28" s="87"/>
-      <c r="H28" s="87"/>
-      <c r="I28" s="87"/>
-      <c r="J28" s="87"/>
-      <c r="K28" s="87"/>
-      <c r="L28" s="87"/>
-      <c r="M28" s="87"/>
-      <c r="N28" s="87"/>
-      <c r="O28" s="87"/>
-      <c r="P28" s="87"/>
-      <c r="Q28" s="87"/>
-      <c r="R28" s="87"/>
-      <c r="S28" s="88"/>
+      <c r="B28" s="110"/>
+      <c r="C28" s="110"/>
+      <c r="D28" s="110"/>
+      <c r="E28" s="110"/>
+      <c r="F28" s="110"/>
+      <c r="G28" s="110"/>
+      <c r="H28" s="110"/>
+      <c r="I28" s="110"/>
+      <c r="J28" s="110"/>
+      <c r="K28" s="110"/>
+      <c r="L28" s="110"/>
+      <c r="M28" s="110"/>
+      <c r="N28" s="110"/>
+      <c r="O28" s="110"/>
+      <c r="P28" s="110"/>
+      <c r="Q28" s="110"/>
+      <c r="R28" s="110"/>
+      <c r="S28" s="110"/>
       <c r="T28" s="12" t="s">
         <v>48</v>
       </c>
@@ -2030,43 +2073,43 @@
       <c r="V28" s="21"/>
     </row>
     <row r="29" spans="1:22" s="6" customFormat="1" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="85" t="s">
+      <c r="A29" s="88" t="s">
         <v>62</v>
       </c>
-      <c r="B29" s="85"/>
-      <c r="C29" s="85"/>
-      <c r="D29" s="85" t="s">
+      <c r="B29" s="88"/>
+      <c r="C29" s="88"/>
+      <c r="D29" s="88" t="s">
         <v>35</v>
       </c>
-      <c r="E29" s="85"/>
-      <c r="F29" s="89" t="s">
+      <c r="E29" s="88"/>
+      <c r="F29" s="88" t="s">
         <v>36</v>
       </c>
-      <c r="G29" s="90"/>
-      <c r="H29" s="85" t="s">
+      <c r="G29" s="88"/>
+      <c r="H29" s="88" t="s">
         <v>63</v>
       </c>
-      <c r="I29" s="85"/>
-      <c r="J29" s="85"/>
-      <c r="K29" s="85" t="s">
+      <c r="I29" s="88"/>
+      <c r="J29" s="88"/>
+      <c r="K29" s="88" t="s">
         <v>37</v>
       </c>
-      <c r="L29" s="85"/>
-      <c r="M29" s="68" t="s">
+      <c r="L29" s="88"/>
+      <c r="M29" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="N29" s="68" t="s">
+      <c r="N29" s="77" t="s">
         <v>39</v>
       </c>
-      <c r="O29" s="85" t="s">
+      <c r="O29" s="88" t="s">
         <v>40</v>
       </c>
-      <c r="P29" s="85"/>
-      <c r="Q29" s="85"/>
-      <c r="R29" s="68" t="s">
+      <c r="P29" s="88"/>
+      <c r="Q29" s="88"/>
+      <c r="R29" s="77" t="s">
         <v>41</v>
       </c>
-      <c r="S29" s="68" t="s">
+      <c r="S29" s="77" t="s">
         <v>42</v>
       </c>
       <c r="T29" s="23" t="s">
@@ -2080,43 +2123,43 @@
       </c>
     </row>
     <row r="30" spans="1:22" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="85">
+      <c r="A30" s="88">
         <v>1</v>
       </c>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85">
+      <c r="B30" s="88"/>
+      <c r="C30" s="88"/>
+      <c r="D30" s="88">
         <v>2</v>
       </c>
-      <c r="E30" s="85"/>
-      <c r="F30" s="89">
+      <c r="E30" s="88"/>
+      <c r="F30" s="88">
         <v>3</v>
       </c>
-      <c r="G30" s="90"/>
-      <c r="H30" s="85">
+      <c r="G30" s="88"/>
+      <c r="H30" s="88">
         <v>4</v>
       </c>
-      <c r="I30" s="85"/>
-      <c r="J30" s="85"/>
-      <c r="K30" s="85">
+      <c r="I30" s="88"/>
+      <c r="J30" s="88"/>
+      <c r="K30" s="88">
         <v>5</v>
       </c>
-      <c r="L30" s="85"/>
-      <c r="M30" s="68">
+      <c r="L30" s="88"/>
+      <c r="M30" s="116">
         <v>6</v>
       </c>
-      <c r="N30" s="68">
+      <c r="N30" s="116">
         <v>7</v>
       </c>
-      <c r="O30" s="85">
+      <c r="O30" s="112">
         <v>8</v>
       </c>
-      <c r="P30" s="85"/>
-      <c r="Q30" s="85"/>
-      <c r="R30" s="68">
+      <c r="P30" s="112"/>
+      <c r="Q30" s="88"/>
+      <c r="R30" s="77">
         <v>9</v>
       </c>
-      <c r="S30" s="68">
+      <c r="S30" s="77">
         <v>10</v>
       </c>
       <c r="T30" s="23" t="s">
@@ -2130,27 +2173,27 @@
       </c>
     </row>
     <row r="31" spans="1:22" s="26" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="77"/>
-      <c r="B31" s="77"/>
-      <c r="C31" s="77"/>
-      <c r="D31" s="77"/>
-      <c r="E31" s="77"/>
-      <c r="F31" s="77"/>
-      <c r="G31" s="77"/>
-      <c r="H31" s="77"/>
-      <c r="I31" s="77"/>
-      <c r="J31" s="77"/>
-      <c r="K31" s="77"/>
-      <c r="L31" s="77"/>
-      <c r="M31" s="80" t="s">
+      <c r="A31" s="113"/>
+      <c r="B31" s="113"/>
+      <c r="C31" s="113"/>
+      <c r="D31" s="113"/>
+      <c r="E31" s="113"/>
+      <c r="F31" s="113"/>
+      <c r="G31" s="113"/>
+      <c r="H31" s="113"/>
+      <c r="I31" s="113"/>
+      <c r="J31" s="113"/>
+      <c r="K31" s="113"/>
+      <c r="L31" s="113"/>
+      <c r="M31" s="117" t="s">
         <v>69</v>
       </c>
-      <c r="N31" s="80"/>
-      <c r="O31" s="80"/>
-      <c r="P31" s="80"/>
-      <c r="Q31" s="111"/>
-      <c r="R31" s="111"/>
-      <c r="S31" s="111"/>
+      <c r="N31" s="118"/>
+      <c r="O31" s="118"/>
+      <c r="P31" s="111"/>
+      <c r="Q31" s="115"/>
+      <c r="R31" s="114"/>
+      <c r="S31" s="114"/>
     </row>
     <row r="32" spans="1:22" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
@@ -2185,13 +2228,13 @@
       <c r="S33" s="26"/>
     </row>
     <row r="34" spans="1:19" s="32" customFormat="1" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="112"/>
-      <c r="B34" s="112"/>
-      <c r="C34" s="112"/>
-      <c r="D34" s="112"/>
-      <c r="E34" s="112"/>
-      <c r="F34" s="112"/>
-      <c r="G34" s="112"/>
+      <c r="A34" s="79"/>
+      <c r="B34" s="79"/>
+      <c r="C34" s="79"/>
+      <c r="D34" s="79"/>
+      <c r="E34" s="79"/>
+      <c r="F34" s="79"/>
+      <c r="G34" s="79"/>
     </row>
     <row r="35" spans="1:19" s="1" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="71"/>
@@ -2215,18 +2258,18 @@
         <v>43</v>
       </c>
       <c r="E37" s="33"/>
-      <c r="F37" s="79"/>
-      <c r="G37" s="79"/>
-      <c r="H37" s="79"/>
-      <c r="I37" s="79"/>
-      <c r="K37" s="81"/>
-      <c r="L37" s="81"/>
-      <c r="M37" s="81"/>
-      <c r="N37" s="81"/>
-      <c r="O37" s="81"/>
-      <c r="P37" s="81"/>
-      <c r="R37" s="82"/>
-      <c r="S37" s="82"/>
+      <c r="F37" s="109"/>
+      <c r="G37" s="109"/>
+      <c r="H37" s="109"/>
+      <c r="I37" s="109"/>
+      <c r="K37" s="107"/>
+      <c r="L37" s="107"/>
+      <c r="M37" s="107"/>
+      <c r="N37" s="107"/>
+      <c r="O37" s="107"/>
+      <c r="P37" s="107"/>
+      <c r="R37" s="87"/>
+      <c r="S37" s="87"/>
     </row>
     <row r="38" spans="1:19" s="7" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="63"/>
@@ -2240,14 +2283,14 @@
       <c r="G38" s="78"/>
       <c r="H38" s="78"/>
       <c r="I38" s="78"/>
-      <c r="K38" s="84" t="s">
+      <c r="K38" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="L38" s="84"/>
-      <c r="M38" s="84"/>
-      <c r="N38" s="84"/>
-      <c r="O38" s="84"/>
-      <c r="P38" s="84"/>
+      <c r="L38" s="86"/>
+      <c r="M38" s="86"/>
+      <c r="N38" s="86"/>
+      <c r="O38" s="86"/>
+      <c r="P38" s="86"/>
       <c r="R38" s="78" t="s">
         <v>46</v>
       </c>
@@ -2276,18 +2319,18 @@
       <c r="D40" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F40" s="83"/>
-      <c r="G40" s="83"/>
-      <c r="H40" s="83"/>
-      <c r="I40" s="83"/>
-      <c r="K40" s="81"/>
-      <c r="L40" s="81"/>
-      <c r="M40" s="81"/>
-      <c r="N40" s="81"/>
-      <c r="O40" s="81"/>
-      <c r="P40" s="81"/>
-      <c r="R40" s="82"/>
-      <c r="S40" s="82"/>
+      <c r="F40" s="108"/>
+      <c r="G40" s="108"/>
+      <c r="H40" s="108"/>
+      <c r="I40" s="108"/>
+      <c r="K40" s="107"/>
+      <c r="L40" s="107"/>
+      <c r="M40" s="107"/>
+      <c r="N40" s="107"/>
+      <c r="O40" s="107"/>
+      <c r="P40" s="107"/>
+      <c r="R40" s="87"/>
+      <c r="S40" s="87"/>
     </row>
     <row r="41" spans="1:19" s="7" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="63"/>
@@ -2301,14 +2344,14 @@
       <c r="G41" s="78"/>
       <c r="H41" s="78"/>
       <c r="I41" s="78"/>
-      <c r="K41" s="84" t="s">
+      <c r="K41" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="L41" s="84"/>
-      <c r="M41" s="84"/>
-      <c r="N41" s="84"/>
-      <c r="O41" s="84"/>
-      <c r="P41" s="84"/>
+      <c r="L41" s="86"/>
+      <c r="M41" s="86"/>
+      <c r="N41" s="86"/>
+      <c r="O41" s="86"/>
+      <c r="P41" s="86"/>
       <c r="R41" s="78" t="s">
         <v>46</v>
       </c>
@@ -2337,6 +2380,68 @@
     </row>
   </sheetData>
   <mergeCells count="78">
+    <mergeCell ref="F38:I38"/>
+    <mergeCell ref="F37:I37"/>
+    <mergeCell ref="M31:P31"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="N37:P37"/>
+    <mergeCell ref="R41:S41"/>
+    <mergeCell ref="R40:S40"/>
+    <mergeCell ref="K40:M40"/>
+    <mergeCell ref="N40:P40"/>
+    <mergeCell ref="F41:I41"/>
+    <mergeCell ref="F40:I40"/>
+    <mergeCell ref="K41:P41"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="A28:S28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:J29"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="O29:Q29"/>
+    <mergeCell ref="O27:P27"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="G27:N27"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="H14:L14"/>
+    <mergeCell ref="H15:L15"/>
+    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="K22:K23"/>
+    <mergeCell ref="L22:L23"/>
+    <mergeCell ref="M22:M23"/>
+    <mergeCell ref="N22:N23"/>
+    <mergeCell ref="S21:S23"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="H16:J16"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="O30:Q30"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="I5:M5"/>
+    <mergeCell ref="I6:M6"/>
+    <mergeCell ref="M12:P12"/>
+    <mergeCell ref="I7:M7"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="B20:S20"/>
+    <mergeCell ref="I21:L21"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="O21:P22"/>
+    <mergeCell ref="Q21:R23"/>
     <mergeCell ref="Q31:S31"/>
     <mergeCell ref="R38:S38"/>
     <mergeCell ref="A34:G34"/>
@@ -2353,68 +2458,6 @@
     <mergeCell ref="A30:C30"/>
     <mergeCell ref="H30:J30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="O30:Q30"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="I5:M5"/>
-    <mergeCell ref="I6:M6"/>
-    <mergeCell ref="M12:P12"/>
-    <mergeCell ref="I7:M7"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="B20:S20"/>
-    <mergeCell ref="I21:L21"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="O21:P22"/>
-    <mergeCell ref="Q21:R23"/>
-    <mergeCell ref="S21:S23"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="H16:J16"/>
-    <mergeCell ref="H18:J18"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="H22:H23"/>
-    <mergeCell ref="I22:I23"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="H14:L14"/>
-    <mergeCell ref="H15:L15"/>
-    <mergeCell ref="J22:J23"/>
-    <mergeCell ref="K22:K23"/>
-    <mergeCell ref="L22:L23"/>
-    <mergeCell ref="M22:M23"/>
-    <mergeCell ref="N22:N23"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="A28:S28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:J29"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="O29:Q29"/>
-    <mergeCell ref="O27:P27"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="G27:N27"/>
-    <mergeCell ref="R41:S41"/>
-    <mergeCell ref="R40:S40"/>
-    <mergeCell ref="K40:M40"/>
-    <mergeCell ref="N40:P40"/>
-    <mergeCell ref="F41:I41"/>
-    <mergeCell ref="F40:I40"/>
-    <mergeCell ref="K41:P41"/>
-    <mergeCell ref="F38:I38"/>
-    <mergeCell ref="F37:I37"/>
-    <mergeCell ref="M31:P31"/>
-    <mergeCell ref="K37:M37"/>
-    <mergeCell ref="N37:P37"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.31496062992125984" top="0.55118110236220474" bottom="0.35433070866141736" header="0.11811023622047245" footer="0.11811023622047245"/>

</xml_diff>